<commit_message>
Modified the conversion page based upon Renee feedback
</commit_message>
<xml_diff>
--- a/_qa/Activity_Tests.xlsx
+++ b/_qa/Activity_Tests.xlsx
@@ -8,8 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_source\Greenshoes\quodsi_lucidchart_package\_qa\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BF2D25A-7F8B-428F-8A8A-7454AB568D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tab Navigation" sheetId="1" r:id="rId1"/>
@@ -22,14 +23,14 @@
     <sheet name="Save-Cancel" sheetId="8" r:id="rId8"/>
     <sheet name="Form Sync" sheetId="9" r:id="rId9"/>
     <sheet name="Edge Cases" sheetId="10" r:id="rId10"/>
-    <sheet name="Model Validation" sheetId="11" r:id="rId14"/>
+    <sheet name="Model Validation" sheetId="11" r:id="rId11"/>
   </sheets>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="390">
   <si>
     <t>Test ID</t>
   </si>
@@ -1220,19 +1221,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color/>
     </font>
   </fonts>
   <fills count="3">
@@ -1260,17 +1262,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="false">
-      <alignment/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1283,7 +1289,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1574,7 +1580,7 @@
     <col min="2" max="2" width="6.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
@@ -1598,7 +1604,7 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -1642,7 +1648,7 @@
       <c r="D2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F2" t="s">
@@ -1662,7 +1668,7 @@
       <c r="D3" t="s">
         <v>17</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F3" t="s">
@@ -1682,7 +1688,7 @@
       <c r="D4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="3" t="s">
         <v>27</v>
       </c>
       <c r="F4" t="s">
@@ -1702,7 +1708,7 @@
       <c r="D5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="3" t="s">
         <v>31</v>
       </c>
       <c r="F5" t="s">
@@ -1722,7 +1728,7 @@
       <c r="D6" t="s">
         <v>17</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="3" t="s">
         <v>35</v>
       </c>
       <c r="F6" t="s">
@@ -1742,7 +1748,7 @@
       <c r="D7" t="s">
         <v>17</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>39</v>
       </c>
       <c r="F7" t="s">
@@ -1924,10 +1930,27 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:N13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="84.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="53" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1940,7 +1963,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -1971,7 +1994,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>331</v>
       </c>
@@ -1984,7 +2007,7 @@
       <c r="D2" t="s">
         <v>333</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>334</v>
       </c>
       <c r="F2" t="s">
@@ -2015,7 +2038,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>337</v>
       </c>
@@ -2028,7 +2051,7 @@
       <c r="D3" t="s">
         <v>339</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="3" t="s">
         <v>340</v>
       </c>
       <c r="F3" t="s">
@@ -2059,7 +2082,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>342</v>
       </c>
@@ -2072,7 +2095,7 @@
       <c r="D4" t="s">
         <v>344</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="3" t="s">
         <v>345</v>
       </c>
       <c r="F4" t="s">
@@ -2103,7 +2126,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>347</v>
       </c>
@@ -2116,7 +2139,7 @@
       <c r="D5" t="s">
         <v>349</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="3" t="s">
         <v>350</v>
       </c>
       <c r="F5" t="s">
@@ -2147,7 +2170,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>352</v>
       </c>
@@ -2160,7 +2183,7 @@
       <c r="D6" t="s">
         <v>354</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="3" t="s">
         <v>355</v>
       </c>
       <c r="F6" t="s">
@@ -2191,7 +2214,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>357</v>
       </c>
@@ -2204,7 +2227,7 @@
       <c r="D7" t="s">
         <v>359</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>360</v>
       </c>
       <c r="F7" t="s">
@@ -2235,7 +2258,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>362</v>
       </c>
@@ -2248,7 +2271,7 @@
       <c r="D8" t="s">
         <v>359</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="3" t="s">
         <v>364</v>
       </c>
       <c r="F8" t="s">
@@ -2279,7 +2302,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>366</v>
       </c>
@@ -2292,7 +2315,7 @@
       <c r="D9" t="s">
         <v>368</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="3" t="s">
         <v>369</v>
       </c>
       <c r="F9" t="s">
@@ -2323,7 +2346,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>371</v>
       </c>
@@ -2336,7 +2359,7 @@
       <c r="D10" t="s">
         <v>373</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="3" t="s">
         <v>374</v>
       </c>
       <c r="F10" t="s">
@@ -2367,7 +2390,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>376</v>
       </c>
@@ -2380,7 +2403,7 @@
       <c r="D11" t="s">
         <v>378</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="3" t="s">
         <v>379</v>
       </c>
       <c r="F11" t="s">
@@ -2411,7 +2434,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>381</v>
       </c>
@@ -2424,7 +2447,7 @@
       <c r="D12" t="s">
         <v>383</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="3" t="s">
         <v>384</v>
       </c>
       <c r="F12" t="s">
@@ -2455,7 +2478,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>386</v>
       </c>
@@ -2468,7 +2491,7 @@
       <c r="D13" t="s">
         <v>285</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="3" t="s">
         <v>388</v>
       </c>
       <c r="F13" t="s">
@@ -2500,6 +2523,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>